<commit_message>
Resultados da última rodada
</commit_message>
<xml_diff>
--- a/compressed_data_classification/src/models/best_models_result/resultados_modelos_reconstructed_2_dot_5.xlsx
+++ b/compressed_data_classification/src/models/best_models_result/resultados_modelos_reconstructed_2_dot_5.xlsx
@@ -476,41 +476,41 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{'mlp__activation': 'identity', 'mlp__alpha': 0.0001, 'mlp__early_stopping': True, 'mlp__hidden_layer_sizes': (15, 10), 'mlp__learning_rate': 'constant', 'mlp__learning_rate_init': 0.001, 'mlp__max_iter': 5000, 'mlp__solver': 'adam'}</t>
+          <t>{'mlp__activation': 'logistic', 'mlp__alpha': 0.001, 'mlp__early_stopping': True, 'mlp__hidden_layer_sizes': (20, 10), 'mlp__learning_rate': 'constant', 'mlp__learning_rate_init': 0.001, 'mlp__max_iter': 5000, 'mlp__solver': 'adam'}</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.8764999999999999</v>
+        <v>0.41</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9932</v>
+        <v>0.9002</v>
       </c>
       <c r="E2" t="n">
-        <v>8.812900000000001</v>
+        <v>44.0359</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
-           0       0.99      0.99      0.99        99
-           1       0.60      0.82      0.69       104
-           2       0.96      0.97      0.97       112
-           3       0.95      1.00      0.97        86
-           4       0.90      0.95      0.93        88
-           5       0.92      0.95      0.93        98
-           6       0.82      0.86      0.84       101
-           7       0.96      0.70      0.81        94
-           8       0.84      0.85      0.84        99
-           9       0.99      1.00      1.00       105
-          10       0.93      0.79      0.85       121
-          11       0.84      0.73      0.78        99
-          12       0.84      0.78      0.81        94
-          13       0.97      0.95      0.96        97
-          14       0.97      0.85      0.91       102
-          15       0.96      0.81      0.88        91
-          16       0.69      0.91      0.79       110
-    accuracy                           0.88      1700
-   macro avg       0.89      0.88      0.88      1700
-weighted avg       0.89      0.88      0.88      1700
+           0       0.39      0.73      0.50        99
+           1       0.22      0.08      0.11       104
+           2       0.25      0.19      0.21       112
+           3       0.27      0.45      0.34        86
+           4       0.15      0.09      0.11        88
+           5       0.31      0.23      0.27        98
+           6       0.71      0.84      0.77       101
+           7       0.28      0.19      0.23        94
+           8       0.12      0.01      0.02        99
+           9       0.95      1.00      0.98       105
+          10       0.69      0.69      0.69       121
+          11       0.22      0.32      0.26        99
+          12       0.37      0.43      0.39        94
+          13       0.36      0.53      0.42        97
+          14       0.38      0.11      0.17       102
+          15       0.43      0.51      0.46        91
+          16       0.33      0.48      0.39       110
+    accuracy                           0.41      1700
+   macro avg       0.38      0.40      0.37      1700
+weighted avg       0.38      0.41      0.38      1700
 </t>
         </is>
       </c>
@@ -518,10 +518,10 @@
         <v>144</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9911</v>
+        <v>0.9049</v>
       </c>
       <c r="I2" t="n">
-        <v>0.002</v>
+        <v>0.0041</v>
       </c>
     </row>
     <row r="3">
@@ -530,41 +530,41 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'svc_rbf__C': 1, 'svc_rbf__gamma': 0.001, 'svc_rbf__kernel': 'rbf', 'svc_rbf__probability': True, 'svc_rbf__random_state': 42}</t>
+          <t>{'svc_rbf__C': 10, 'svc_rbf__gamma': 0.001, 'svc_rbf__kernel': 'rbf', 'svc_rbf__probability': True, 'svc_rbf__random_state': 42}</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.9335</v>
+        <v>0.4735</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9972</v>
+        <v>0.9036</v>
       </c>
       <c r="E3" t="n">
-        <v>3.2682</v>
+        <v>33.1</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
-           0       0.99      1.00      0.99        99
-           1       0.93      0.97      0.95       104
-           2       0.98      0.99      0.99       112
-           3       1.00      0.97      0.98        86
-           4       0.93      0.93      0.93        88
-           5       0.95      0.93      0.94        98
-           6       0.98      0.91      0.94       101
-           7       0.99      0.86      0.92        94
-           8       0.82      0.91      0.86        99
-           9       1.00      1.00      1.00       105
-          10       0.97      0.98      0.98       121
-          11       0.97      0.85      0.90        99
-          12       0.69      0.87      0.77        94
-          13       0.99      1.00      0.99        97
-          14       1.00      0.93      0.96       102
-          15       0.92      0.77      0.84        91
-          16       0.86      0.95      0.91       110
-    accuracy                           0.93      1700
-   macro avg       0.94      0.93      0.93      1700
-weighted avg       0.94      0.93      0.93      1700
+           0       0.82      0.95      0.88        99
+           1       0.35      0.26      0.30       104
+           2       0.51      0.38      0.44       112
+           3       0.42      0.34      0.37        86
+           4       0.22      0.23      0.22        88
+           5       0.25      0.19      0.22        98
+           6       0.89      0.77      0.83       101
+           7       0.40      0.27      0.32        94
+           8       0.25      0.17      0.20        99
+           9       0.99      1.00      1.00       105
+          10       0.79      0.70      0.74       121
+          11       0.37      0.22      0.28        99
+          12       0.22      0.21      0.21        94
+          13       0.85      0.71      0.78        97
+          14       0.25      0.17      0.20       102
+          15       0.17      0.65      0.27        91
+          16       0.65      0.69      0.67       110
+    accuracy                           0.47      1700
+   macro avg       0.49      0.47      0.47      1700
+weighted avg       0.51      0.47      0.48      1700
 </t>
         </is>
       </c>
@@ -572,10 +572,10 @@
         <v>9</v>
       </c>
       <c r="H3" t="n">
-        <v>0.9963</v>
+        <v>0.9082</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0011</v>
+        <v>0.0033</v>
       </c>
     </row>
     <row r="4">
@@ -588,37 +588,37 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9341</v>
+        <v>0.2835</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9974</v>
+        <v>0.8658</v>
       </c>
       <c r="E4" t="n">
-        <v>4.7324</v>
+        <v>33.7624</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
-           0       0.97      1.00      0.99        99
-           1       0.96      0.85      0.90       104
-           2       0.97      0.99      0.98       112
-           3       0.99      1.00      0.99        86
-           4       0.95      0.99      0.97        88
-           5       0.98      0.96      0.97        98
-           6       0.91      0.94      0.93       101
-           7       0.99      0.76      0.86        94
-           8       0.80      0.91      0.85        99
-           9       0.99      1.00      1.00       105
-          10       0.95      0.93      0.94       121
-          11       0.93      0.94      0.93        99
-          12       0.96      0.85      0.90        94
-          13       0.99      1.00      0.99        97
-          14       1.00      0.95      0.97       102
-          15       0.95      0.88      0.91        91
-          16       0.72      0.94      0.81       110
-    accuracy                           0.93      1700
-   macro avg       0.94      0.93      0.94      1700
-weighted avg       0.94      0.93      0.93      1700
+           0       0.22      0.10      0.14        99
+           1       0.29      0.22      0.25       104
+           2       0.22      0.06      0.10       112
+           3       0.29      0.33      0.31        86
+           4       0.25      0.06      0.09        88
+           5       0.32      0.31      0.31        98
+           6       0.80      0.82      0.81       101
+           7       0.18      0.26      0.21        94
+           8       0.76      0.13      0.22        99
+           9       0.19      1.00      0.31       105
+          10       0.39      0.16      0.22       121
+          11       0.33      0.24      0.28        99
+          12       0.78      0.22      0.35        94
+          13       0.20      0.56      0.29        97
+          14       0.00      0.00      0.00       102
+          15       0.38      0.40      0.39        91
+          16       0.00      0.00      0.00       110
+    accuracy                           0.28      1700
+   macro avg       0.33      0.29      0.25      1700
+weighted avg       0.33      0.28      0.25      1700
 </t>
         </is>
       </c>
@@ -626,10 +626,10 @@
         <v>5</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9971</v>
+        <v>0.8615</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0005</v>
+        <v>0.0046</v>
       </c>
     </row>
   </sheetData>

</xml_diff>